<commit_message>
Updated dataset with corrected version
</commit_message>
<xml_diff>
--- a/data/Category_Names.xlsx
+++ b/data/Category_Names.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8caa5b9871172da9/Desktop/grocery-classification/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="11_AD4DB114E441178AC67DF4600ED0F2F4683EDF26" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB669B3E-EFBD-4F7F-8863-700F9D5ED5B2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56141242-E9B7-414B-9F84-62A8B12D9CD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="71">
   <si>
     <t>TOTAL MARKET</t>
   </si>
@@ -237,16 +237,13 @@
     <t>Pet Snacks Mix</t>
   </si>
   <si>
-    <t>Label</t>
+    <t>Original Predictions</t>
   </si>
   <si>
     <t>Other</t>
   </si>
   <si>
     <t>Food</t>
-  </si>
-  <si>
-    <t>Drink</t>
   </si>
   <si>
     <t>Drinks</t>
@@ -752,7 +749,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
@@ -760,7 +757,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
@@ -768,7 +765,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
@@ -776,7 +773,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
@@ -784,7 +781,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
@@ -792,7 +789,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
@@ -800,7 +797,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
@@ -808,7 +805,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
@@ -816,7 +813,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
@@ -1000,7 +997,7 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">
@@ -1016,7 +1013,7 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.3">
@@ -1024,7 +1021,7 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.3">
@@ -1032,7 +1029,7 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.3">
@@ -1040,7 +1037,7 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.3">
@@ -1048,7 +1045,7 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.3">
@@ -1056,7 +1053,7 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.3">
@@ -1064,7 +1061,7 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.3">
@@ -1072,7 +1069,7 @@
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
@@ -1080,7 +1077,7 @@
         <v>53</v>
       </c>
       <c r="B54" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
@@ -1088,7 +1085,7 @@
         <v>54</v>
       </c>
       <c r="B55" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
@@ -1096,7 +1093,7 @@
         <v>55</v>
       </c>
       <c r="B56" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
@@ -1104,7 +1101,7 @@
         <v>56</v>
       </c>
       <c r="B57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
@@ -1112,7 +1109,7 @@
         <v>57</v>
       </c>
       <c r="B58" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
@@ -1120,7 +1117,7 @@
         <v>58</v>
       </c>
       <c r="B59" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
@@ -1128,7 +1125,7 @@
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
@@ -1136,7 +1133,7 @@
         <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
@@ -1144,7 +1141,7 @@
         <v>61</v>
       </c>
       <c r="B62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
@@ -1152,7 +1149,7 @@
         <v>62</v>
       </c>
       <c r="B63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
@@ -1160,7 +1157,7 @@
         <v>63</v>
       </c>
       <c r="B64" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>